<commit_message>
Aura: superficie 73 m² según presupuesto SIPCOR
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PL4fade9uMUQLM1tmUvUUs
</commit_message>
<xml_diff>
--- a/URBANSIP/AURA/Aura_Revision_Costo_30-09-26.xlsx
+++ b/URBANSIP/AURA/Aura_Revision_Costo_30-09-26.xlsx
@@ -70,7 +70,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -92,11 +92,55 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +170,8 @@
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -525,11 +571,11 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Superficie cubierta que se vende (ficha)</t>
+          <t>Superficie cubierta (presupuesto SIPCOR #2790, 08/09/26)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5">
@@ -730,8 +776,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
@@ -769,7 +813,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -915,7 +958,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
@@ -937,6 +979,10 @@
           <t>Está en el Excel de materiales ($850.000 + $3.240.000) y la planilla de mano de obra también tiene días de instalaciones. Puede estar contada dos veces (≈ USD 2.640).</t>
         </is>
       </c>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="21" t="n"/>
+      <c r="G10" s="22" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -949,9 +995,13 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>El Excel de costos divide por 78 m²; la ficha vende 72 m², la planilla de mano de obra usa 72 y el presupuesto SIPCOR dice 73 m². Con 72 m² el costo por m² sube un 8%.</t>
-        </is>
-      </c>
+          <t>Definido: 73 m² cubiertos (presupuesto SIPCOR #2790). El Excel de costos usaba 78 m² y la ficha y la planilla de mano de obra, 72 m². Hay que corregir la ficha.</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="22" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -967,6 +1017,10 @@
           <t>La ficha dice cubierta SIP EPS 50 mm; el Excel cotiza cabios de pino + chapa. Confirmar que los paneles de techo están dentro del kit de $26,9 M.</t>
         </is>
       </c>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1281,7 +1335,6 @@
       </c>
       <c r="E13" s="20" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="D15" s="8" t="inlineStr">
         <is>
@@ -1320,7 +1373,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -1519,7 +1571,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>

</xml_diff>